<commit_message>
📊 BIST Screener | 07.04.2026 16:30 | 605 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-07.xlsx
+++ b/data/bist_screener_2026-04-07.xlsx
@@ -25619,21 +25619,21 @@
     <row r="579">
       <c r="A579" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B579" s="7" t="n">
-        <v>168.4</v>
+        <v>2.94</v>
       </c>
       <c r="C579" s="8" t="n">
-        <v>0.0256</v>
+        <v>-0.04849999999999999</v>
       </c>
       <c r="D579" s="9" t="n">
-        <v>15470000</v>
+        <v>270290000</v>
       </c>
       <c r="E579" s="6" t="inlineStr"/>
       <c r="F579" s="7" t="n">
-        <v>78.06</v>
+        <v>63.92</v>
       </c>
       <c r="G579" s="6" t="inlineStr"/>
       <c r="H579" s="6" t="inlineStr"/>
@@ -25641,12 +25641,12 @@
       <c r="J579" s="6" t="inlineStr"/>
       <c r="K579" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L579" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M579" s="6" t="inlineStr"/>
@@ -25654,42 +25654,36 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>16.58</v>
+        <v>7</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>-0.027</v>
+        <v>-0.0141</v>
       </c>
       <c r="D580" s="5" t="n">
-        <v>11820000</v>
+        <v>10720000</v>
       </c>
       <c r="E580" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.28</v>
       </c>
       <c r="F580" s="3" t="n">
-        <v>39.94</v>
-      </c>
-      <c r="G580" s="3" t="n">
-        <v>156.71</v>
-      </c>
+        <v>35.17</v>
+      </c>
+      <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
-      <c r="I580" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J580" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I580" s="2" t="inlineStr"/>
+      <c r="J580" s="2" t="inlineStr"/>
       <c r="K580" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L580" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M580" s="2" t="inlineStr"/>
@@ -25697,40 +25691,38 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>146.4</v>
+        <v>59.75</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>0.0999</v>
+        <v>-0.0409</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>730480</v>
+        <v>988710</v>
       </c>
       <c r="E581" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F581" s="7" t="n">
-        <v>71.69</v>
+        <v>52.24</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
-      <c r="I581" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
+      <c r="I581" s="6" t="inlineStr"/>
       <c r="J581" s="8" t="n">
-        <v>-0.4897</v>
+        <v>0.4139</v>
       </c>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L581" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M581" s="6" t="inlineStr"/>
@@ -25738,58 +25730,48 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>58.15</v>
+        <v>81.2</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>-0.0219</v>
+        <v>-0.0089</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>3410000</v>
+        <v>12220000</v>
       </c>
       <c r="E582" s="2" t="inlineStr"/>
       <c r="F582" s="3" t="n">
-        <v>44.17</v>
+        <v>39.33</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
       <c r="I582" s="2" t="inlineStr"/>
       <c r="J582" s="2" t="inlineStr"/>
-      <c r="K582" s="2" t="inlineStr">
-        <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L582" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+      <c r="K582" s="2" t="inlineStr"/>
+      <c r="L582" s="2" t="inlineStr"/>
       <c r="M582" s="2" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>26.98</v>
+        <v>168.4</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.0182</v>
+        <v>0.0256</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>12720000</v>
-      </c>
-      <c r="E583" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>15470000</v>
+      </c>
+      <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>51.22</v>
+        <v>78.06</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25797,12 +25779,12 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25810,21 +25792,21 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>23.22</v>
+        <v>13.59</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0421</v>
+        <v>-0.0755</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>18100000</v>
+        <v>77330000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>53.02</v>
+        <v>53.82</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25832,12 +25814,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25845,36 +25827,42 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>3.15</v>
+        <v>16.58</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.1</v>
+        <v>-0.027</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>57800000</v>
+        <v>11820000</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.9246</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>52.54</v>
-      </c>
-      <c r="G585" s="6" t="inlineStr"/>
+        <v>39.94</v>
+      </c>
+      <c r="G585" s="7" t="n">
+        <v>156.71</v>
+      </c>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="6" t="inlineStr"/>
+      <c r="I585" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J585" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25882,21 +25870,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>40.88</v>
+        <v>58.15</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.039</v>
+        <v>-0.0219</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>26340000</v>
+        <v>3410000</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>55.56</v>
+        <v>44.17</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25904,12 +25892,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25917,73 +25905,71 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>201.1</v>
+        <v>8.15</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0441</v>
+        <v>-0.0355</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>7370000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>210530</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>71.23</v>
+        <v>41.77</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr"/>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>2.72</v>
+        <v>35</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0073</v>
+        <v>-0.0374</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>89900000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.6898000000000001</v>
-      </c>
+        <v>5290000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>44.48</v>
+        <v>42.43</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>-2.0083</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25991,62 +25977,42 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="C589" s="8" t="n">
-        <v>-0.0365</v>
-      </c>
-      <c r="D589" s="9" t="n">
-        <v>67370000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.7119</v>
-      </c>
-      <c r="F589" s="7" t="n">
-        <v>63.76</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="C589" s="6" t="inlineStr"/>
+      <c r="D589" s="6" t="inlineStr"/>
+      <c r="E589" s="6" t="inlineStr"/>
+      <c r="F589" s="6" t="inlineStr"/>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
-      <c r="K589" s="6" t="inlineStr">
-        <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
+      <c r="K589" s="6" t="inlineStr"/>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>ZGYO</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>15.8</v>
+        <v>26.68</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.08740000000000001</v>
+        <v>-0.0213</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>111910000</v>
+        <v>19790000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>88.31999999999999</v>
+        <v>53.32</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26067,38 +26033,38 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>59.75</v>
+        <v>2.72</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0409</v>
+        <v>-0.0073</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>988710</v>
+        <v>89900000</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.6898000000000001</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>52.24</v>
+        <v>44.48</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="8" t="n">
-        <v>0.4139</v>
+        <v>-2.0083</v>
       </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26106,95 +26072,113 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>81.2</v>
+        <v>26.98</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0089</v>
+        <v>-0.0182</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>12220000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>12720000</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>39.33</v>
+        <v>51.22</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
       <c r="J592" s="2" t="inlineStr"/>
-      <c r="K592" s="2" t="inlineStr"/>
-      <c r="L592" s="2" t="inlineStr"/>
+      <c r="K592" s="2" t="inlineStr">
+        <is>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>8.15</v>
+        <v>3</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0355</v>
+        <v>-0.0066</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>210530</v>
+        <v>25850000</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.95</v>
+        <v>0.1672</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>41.77</v>
+        <v>53.9</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-5.3262</v>
       </c>
       <c r="J593" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.2562</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>235</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0432</v>
+        <v>-0.0098</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>8950</v>
+        <v>23900</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.58</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>34.99</v>
+        <v>40.33</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr"/>
@@ -26203,21 +26187,21 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>33.16</v>
+        <v>40.88</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0141</v>
+        <v>-0.039</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>5200000</v>
+        <v>26340000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>54.6</v>
+        <v>55.56</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26225,12 +26209,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26238,36 +26222,38 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0141</v>
+        <v>-0.0922</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>10720000</v>
+        <v>137550000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.28</v>
+        <v>0.2478</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>35.17</v>
+        <v>14.49</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26275,38 +26261,34 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>6.5</v>
+        <v>33.16</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0922</v>
+        <v>0.0141</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>137550000</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.2478</v>
-      </c>
+        <v>5200000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>14.49</v>
+        <v>54.6</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26314,40 +26296,40 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>3</v>
+        <v>3.17</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0066</v>
+        <v>-0.0365</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>25850000</v>
+        <v>67370000</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.7119</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>53.9</v>
+        <v>63.76</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="4" t="n">
-        <v>-5.3262</v>
+        <v>-191.6342</v>
       </c>
       <c r="J598" s="4" t="n">
-        <v>-4.2562</v>
+        <v>-0.8093</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26355,21 +26337,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>13.59</v>
+        <v>6.15</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0755</v>
+        <v>0.0389</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>77330000</v>
+        <v>13750000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>53.82</v>
+        <v>83.29000000000001</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26377,55 +26359,67 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>171</v>
-      </c>
-      <c r="C600" s="2" t="inlineStr"/>
-      <c r="D600" s="2" t="inlineStr"/>
+        <v>15.8</v>
+      </c>
+      <c r="C600" s="4" t="n">
+        <v>0.08740000000000001</v>
+      </c>
+      <c r="D600" s="5" t="n">
+        <v>111910000</v>
+      </c>
       <c r="E600" s="2" t="inlineStr"/>
-      <c r="F600" s="2" t="inlineStr"/>
+      <c r="F600" s="3" t="n">
+        <v>88.31999999999999</v>
+      </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
       <c r="J600" s="2" t="inlineStr"/>
-      <c r="K600" s="2" t="inlineStr"/>
-      <c r="L600" s="2" t="inlineStr"/>
+      <c r="K600" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>35</v>
+        <v>3.15</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0374</v>
+        <v>-0.1</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>5290000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>57800000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>42.43</v>
+        <v>52.54</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26433,12 +26427,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26446,21 +26440,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>6.15</v>
+        <v>18.4</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0389</v>
+        <v>-0.0387</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>13750000</v>
+        <v>118280000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>83.29000000000001</v>
+        <v>60.16</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26471,77 +26465,85 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>85.84999999999999</v>
+        <v>201.1</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0098</v>
+        <v>0.0441</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>23900</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>7370000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>40.33</v>
+        <v>71.23</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>18.4</v>
+        <v>146.4</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0387</v>
+        <v>0.0999</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>118280000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>730480</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>60.16</v>
+        <v>71.69</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26549,21 +26551,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>2.94</v>
+        <v>23.22</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.04849999999999999</v>
+        <v>-0.0421</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>270290000</v>
+        <v>18100000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>63.92</v>
+        <v>53.02</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26571,12 +26573,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26584,21 +26586,23 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>ZGYO</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>26.68</v>
+        <v>235</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0213</v>
+        <v>-0.0432</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>19790000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>8950</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>53.32</v>
+        <v>34.99</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26606,14 +26610,10 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26638,7 +26638,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>07.04.2026 15:30</t>
+          <t>07.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 07.04.2026 18:14 | 605 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-07.xlsx
+++ b/data/bist_screener_2026-04-07.xlsx
@@ -25619,63 +25619,69 @@
     <row r="579">
       <c r="A579" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B579" s="7" t="n">
-        <v>2.94</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="C579" s="8" t="n">
-        <v>-0.04849999999999999</v>
+        <v>-0.0098</v>
       </c>
       <c r="D579" s="9" t="n">
-        <v>270290000</v>
-      </c>
-      <c r="E579" s="6" t="inlineStr"/>
+        <v>23900</v>
+      </c>
+      <c r="E579" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F579" s="7" t="n">
-        <v>63.92</v>
+        <v>40.33</v>
       </c>
       <c r="G579" s="6" t="inlineStr"/>
       <c r="H579" s="6" t="inlineStr"/>
-      <c r="I579" s="6" t="inlineStr"/>
-      <c r="J579" s="6" t="inlineStr"/>
+      <c r="I579" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J579" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K579" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L579" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L579" s="6" t="inlineStr"/>
       <c r="M579" s="6" t="inlineStr"/>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>-0.0141</v>
+        <v>-0.0066</v>
       </c>
       <c r="D580" s="5" t="n">
-        <v>10720000</v>
+        <v>25850000</v>
       </c>
       <c r="E580" s="4" t="n">
-        <v>0.28</v>
+        <v>0.1672</v>
       </c>
       <c r="F580" s="3" t="n">
-        <v>35.17</v>
+        <v>53.9</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
-      <c r="I580" s="2" t="inlineStr"/>
-      <c r="J580" s="2" t="inlineStr"/>
+      <c r="I580" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J580" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K580" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -25683,7 +25689,7 @@
       </c>
       <c r="L580" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M580" s="2" t="inlineStr"/>
@@ -25691,38 +25697,36 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>59.75</v>
+        <v>3.15</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>-0.0409</v>
+        <v>-0.1</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>988710</v>
+        <v>57800000</v>
       </c>
       <c r="E581" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.8667</v>
       </c>
       <c r="F581" s="7" t="n">
-        <v>52.24</v>
+        <v>52.54</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
       <c r="I581" s="6" t="inlineStr"/>
-      <c r="J581" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J581" s="6" t="inlineStr"/>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L581" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M581" s="6" t="inlineStr"/>
@@ -25730,139 +25734,131 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>81.2</v>
+        <v>201.1</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>-0.0089</v>
+        <v>0.0441</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>12220000</v>
+        <v>7370000</v>
       </c>
       <c r="E582" s="2" t="inlineStr"/>
       <c r="F582" s="3" t="n">
-        <v>39.33</v>
+        <v>71.23</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
       <c r="I582" s="2" t="inlineStr"/>
       <c r="J582" s="2" t="inlineStr"/>
-      <c r="K582" s="2" t="inlineStr"/>
-      <c r="L582" s="2" t="inlineStr"/>
+      <c r="K582" s="2" t="inlineStr">
+        <is>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L582" s="2" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M582" s="2" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>168.4</v>
+        <v>8.15</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0256</v>
+        <v>-0.0355</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>15470000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
+        <v>210530</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F583" s="7" t="n">
-        <v>78.06</v>
+        <v>41.77</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>13.59</v>
-      </c>
-      <c r="C584" s="4" t="n">
-        <v>-0.0755</v>
-      </c>
-      <c r="D584" s="5" t="n">
-        <v>77330000</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="C584" s="2" t="inlineStr"/>
+      <c r="D584" s="2" t="inlineStr"/>
       <c r="E584" s="2" t="inlineStr"/>
-      <c r="F584" s="3" t="n">
-        <v>53.82</v>
-      </c>
+      <c r="F584" s="2" t="inlineStr"/>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
       <c r="J584" s="2" t="inlineStr"/>
-      <c r="K584" s="2" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L584" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="K584" s="2" t="inlineStr"/>
+      <c r="L584" s="2" t="inlineStr"/>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>16.58</v>
+        <v>6.5</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.027</v>
+        <v>-0.0922</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>11820000</v>
+        <v>137550000</v>
       </c>
       <c r="E585" s="8" t="n">
-        <v>0.9246</v>
+        <v>0.2478</v>
       </c>
       <c r="F585" s="7" t="n">
-        <v>39.94</v>
-      </c>
-      <c r="G585" s="7" t="n">
-        <v>156.71</v>
-      </c>
+        <v>14.49</v>
+      </c>
+      <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J585" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25870,34 +25866,40 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>58.15</v>
+        <v>3.17</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0219</v>
+        <v>-0.0365</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>3410000</v>
-      </c>
-      <c r="E586" s="2" t="inlineStr"/>
+        <v>67370000</v>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F586" s="3" t="n">
-        <v>44.17</v>
+        <v>63.76</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="2" t="inlineStr"/>
-      <c r="J586" s="2" t="inlineStr"/>
+      <c r="I586" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J586" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25905,114 +25907,114 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>8.15</v>
+        <v>33.16</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0355</v>
+        <v>0.0141</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>210530</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>5200000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>41.77</v>
+        <v>54.6</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>35</v>
+        <v>81.2</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0374</v>
+        <v>-0.0089</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>5290000</v>
+        <v>12220000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>42.43</v>
+        <v>39.33</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr">
-        <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+      <c r="K588" s="2" t="inlineStr"/>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>171</v>
-      </c>
-      <c r="C589" s="6" t="inlineStr"/>
-      <c r="D589" s="6" t="inlineStr"/>
+        <v>6.15</v>
+      </c>
+      <c r="C589" s="8" t="n">
+        <v>0.0389</v>
+      </c>
+      <c r="D589" s="9" t="n">
+        <v>13750000</v>
+      </c>
       <c r="E589" s="6" t="inlineStr"/>
-      <c r="F589" s="6" t="inlineStr"/>
+      <c r="F589" s="7" t="n">
+        <v>83.29000000000001</v>
+      </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
       <c r="I589" s="6" t="inlineStr"/>
       <c r="J589" s="6" t="inlineStr"/>
-      <c r="K589" s="6" t="inlineStr"/>
+      <c r="K589" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
       <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ZGYO</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>26.68</v>
+        <v>168.4</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0213</v>
+        <v>0.0256</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>19790000</v>
+        <v>15470000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>53.32</v>
+        <v>78.06</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26020,12 +26022,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26033,38 +26035,34 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>2.72</v>
+        <v>35</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0073</v>
+        <v>-0.0374</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>89900000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.6898000000000001</v>
-      </c>
+        <v>5290000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>44.48</v>
+        <v>42.43</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="8" t="n">
-        <v>-2.0083</v>
-      </c>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26072,23 +26070,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>26.98</v>
+        <v>23.22</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0182</v>
+        <v>-0.0421</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>12720000</v>
-      </c>
-      <c r="E592" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>18100000</v>
+      </c>
+      <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>51.22</v>
+        <v>53.02</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26096,12 +26092,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26109,99 +26105,89 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>3</v>
+        <v>235</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0066</v>
+        <v>-0.0432</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>25850000</v>
+        <v>8950</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2578</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>53.9</v>
+        <v>34.99</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>85.84999999999999</v>
+        <v>58.15</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0098</v>
+        <v>-0.0219</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>23900</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>3410000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>40.33</v>
+        <v>44.17</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>40.88</v>
+        <v>15.8</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.039</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>26340000</v>
+        <v>111910000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>55.56</v>
+        <v>88.31999999999999</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26209,12 +26195,12 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26222,38 +26208,34 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.5</v>
+        <v>40.88</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0922</v>
+        <v>-0.039</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>137550000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.2478</v>
-      </c>
+        <v>26340000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>14.49</v>
+        <v>55.56</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26261,21 +26243,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>33.16</v>
+        <v>13.59</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0141</v>
+        <v>-0.0755</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>5200000</v>
+        <v>77330000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>54.6</v>
+        <v>53.82</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26283,12 +26265,12 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M597" s="6" t="inlineStr"/>
@@ -26296,40 +26278,40 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>3.17</v>
+        <v>146.4</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0365</v>
+        <v>0.0999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>67370000</v>
+        <v>730480</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.7119</v>
+        <v>0.1071</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>63.76</v>
+        <v>71.69</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="4" t="n">
-        <v>-191.6342</v>
+        <v>-3.6635</v>
       </c>
       <c r="J598" s="4" t="n">
-        <v>-0.8093</v>
+        <v>-0.4897</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26337,21 +26319,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>6.15</v>
+        <v>2.94</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0389</v>
+        <v>-0.04849999999999999</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>13750000</v>
+        <v>270290000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>83.29000000000001</v>
+        <v>63.92</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26362,40 +26344,48 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>15.8</v>
+        <v>2.72</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.08740000000000001</v>
+        <v>-0.0073</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>111910000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>89900000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.6898000000000001</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>88.31999999999999</v>
+        <v>44.48</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="J600" s="4" t="n">
+        <v>-2.0083</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26403,36 +26393,42 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>3.15</v>
+        <v>16.58</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.1</v>
+        <v>-0.027</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>57800000</v>
+        <v>11820000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.9246</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>52.54</v>
-      </c>
-      <c r="G601" s="6" t="inlineStr"/>
+        <v>39.94</v>
+      </c>
+      <c r="G601" s="7" t="n">
+        <v>156.71</v>
+      </c>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26440,34 +26436,38 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>18.4</v>
+        <v>59.75</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0387</v>
+        <v>-0.0409</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>118280000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>988710</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>60.16</v>
+        <v>52.24</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="J602" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26475,21 +26475,21 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>ZGYO</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>201.1</v>
+        <v>26.68</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0441</v>
+        <v>-0.0213</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>7370000</v>
+        <v>19790000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>71.23</v>
+        <v>53.32</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26497,12 +26497,12 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26510,40 +26510,36 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>146.4</v>
+        <v>7</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0999</v>
+        <v>-0.0141</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>730480</v>
+        <v>10720000</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.28</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>71.69</v>
+        <v>35.17</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26551,21 +26547,21 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>23.22</v>
+        <v>18.4</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0421</v>
+        <v>-0.0387</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>18100000</v>
+        <v>118280000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>53.02</v>
+        <v>60.16</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
@@ -26573,12 +26569,12 @@
       <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26586,23 +26582,23 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>235</v>
+        <v>26.98</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0432</v>
+        <v>-0.0182</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>8950</v>
+        <v>12720000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.2667</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>34.99</v>
+        <v>51.22</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26610,10 +26606,14 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26638,7 +26638,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>07.04.2026 16:30</t>
+          <t>07.04.2026 18:14</t>
         </is>
       </c>
     </row>

</xml_diff>